<commit_message>
Housekeeping de datos + constructor de base histórica corregido
- Fuentes actualizadas por el pipeline (costos, cache de proyección,
  consolidado de salidas, proyecciones de compra) y nuevas descargas de
  historial de Contabilium (15-21/07).
- construir_base_historica.py: la tabla proyeccion/proyeccion_mensual
  ahora toma data_proyeccion.js (publicado, con el saldo_stock ya
  corregido) en vez de Analisis_proyeccion_cache.json (forecast crudo sin
  los overrides del mes en curso) — si no, la base quedaba con el saldo
  viejo pese al fix de actualizar_bosquegin.py. Se agregan también
  venta_prom_6m/12m y proyeccion_mensual, que sólo están en el publicado.
</commit_message>
<xml_diff>
--- a/Data/Supply Chain/proyecciones/proyecciones.xlsx
+++ b/Data/Supply Chain/proyecciones/proyecciones.xlsx
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>23.8</v>
+        <v>24.2</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0</v>
@@ -563,7 +563,7 @@
         <v>48</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>83</v>
@@ -594,19 +594,19 @@
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.9</v>
+        <v>21.9</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
@@ -635,19 +635,19 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>27.9</v>
+        <v>27.1</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>57</v>
@@ -680,19 +680,19 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>22.5</v>
+        <v>26.4</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
@@ -718,22 +718,22 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>198</v>
+        <v>24</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1737.5</v>
+        <v>1809.7</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1540</v>
+        <v>1786</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3277</v>
+        <v>3595</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>5014</v>
+        <v>5405</v>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1200</v>
+        <v>1008</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>7121.9</v>
+        <v>6791.6</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>5922</v>
+        <v>5784</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>13044</v>
+        <v>12575</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>20166</v>
+        <v>19367</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>4800</v>
@@ -853,22 +853,22 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1184</v>
+        <v>980</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1979</v>
+        <v>1978.5</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>795</v>
+        <v>998</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>2774</v>
+        <v>2977</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4753</v>
+        <v>4956</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>2025</v>
@@ -878,97 +878,97 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>600009</v>
+        <v>110027</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>VASO FERIADO 400 ML</t>
+          <t>CERVEZA TEMPLE WOLF IPA 0% ALCOHOL 473 ML</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>CRISTALERIA</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>VIDRIO TANGO</t>
+          <t>CERVEZAS</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>36</v>
+        <v>678</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>38.2</v>
+        <v>788.8</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0.9</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>2</v>
+        <v>111</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>40</v>
+        <v>900</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>79</v>
+        <v>1688</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>110005</v>
+        <v>600009</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA TEMPLE BLACK SOUL STOUT 473 ML</t>
+          <t>VASO FERIADO 400 ML</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>CRISTALERIA</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>CERVEZAS</t>
+          <t>VIDRIO TANGO</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>0.9</v>
+        <v>36.1</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="K11" s="2" t="n">
         <v>7</v>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K11" s="2" t="n">
-        <v>18</v>
       </c>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>110027</v>
+        <v>110005</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA TEMPLE WOLF IPA 0% ALCOHOL 473 ML</t>
+          <t>CERVEZA TEMPLE BLACK SOUL STOUT 473 ML</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -982,25 +982,25 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>858</v>
+        <v>6</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>780</v>
+        <v>4.9</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>702</v>
+        <v>4</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1482</v>
+        <v>9</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
@@ -1025,22 +1025,22 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>606</v>
+        <v>554</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>424.5</v>
+        <v>424.2</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>668</v>
+        <v>719</v>
       </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
@@ -1048,11 +1048,11 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>100017</v>
+        <v>100004</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FERIADO ROJO VERMU BARRIL 20 LTS</t>
+          <t>FERIADO ROJO VERMÚ 750 ML</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1066,36 +1066,36 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>19</v>
+        <v>2026</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>1.9</v>
+        <v>1036.1</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>10</v>
+        <v>1082</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>10</v>
+        <v>591</v>
       </c>
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>100004</v>
+        <v>100017</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>FERIADO ROJO VERMÚ 750 ML</t>
+          <t>FERIADO ROJO VERMU BARRIL 20 LTS</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1109,10 +1109,10 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2092</v>
+        <v>19</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1048.2</v>
+        <v>9.6</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2</v>
@@ -1121,13 +1121,13 @@
         <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1053</v>
+        <v>10</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>591</v>
+        <v>10</v>
       </c>
       <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
@@ -1152,13 +1152,13 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>763</v>
+        <v>715</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>348.2</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>282</v>
+        <v>330</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
@@ -1175,31 +1175,31 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>500019</v>
+        <v>100003</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GIFT PACK NATIVO</t>
+          <t>GIN BOSQUE REFUGIOS BOTELLA 500 ML</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>COMBO</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>GIFT PACK</t>
+          <t>GIN</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>6</v>
+        <v>212</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>2.1</v>
+        <v>75</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>0</v>
@@ -1208,7 +1208,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
@@ -1216,28 +1216,28 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>100003</v>
+        <v>500019</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>GIN BOSQUE REFUGIOS BOTELLA 500 ML</t>
+          <t>GIFT PACK NATIVO</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>GIN</t>
+          <t>GIFT PACK</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>220</v>
+        <v>6</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>74.8</v>
+        <v>2.1</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>2.9</v>
@@ -1249,7 +1249,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>

</xml_diff>

<commit_message>
Housekeeping de datos del pipeline
Costos/destilería CSV, consolidado de salidas, proyecciones de compra,
caché de última fecha de historial, y nueva descarga de Contabilium
(21-23/07).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Supply Chain/proyecciones/proyecciones.xlsx
+++ b/Data/Supply Chain/proyecciones/proyecciones.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>24.2</v>
+        <v>24.4</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0</v>
@@ -560,7 +560,7 @@
         <v>24</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>73</v>
@@ -594,19 +594,19 @@
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>21.9</v>
+        <v>19.2</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
@@ -635,7 +635,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -680,19 +680,19 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>26.4</v>
+        <v>27.6</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
@@ -721,19 +721,19 @@
         <v>24</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1809.7</v>
+        <v>1828</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1786</v>
+        <v>1804</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>3595</v>
+        <v>3632</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>5405</v>
+        <v>5460</v>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1008</v>
+        <v>42</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>6791.6</v>
+        <v>6824</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>5784</v>
+        <v>6782</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>12575</v>
+        <v>13606</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>19367</v>
+        <v>20430</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>4800</v>
@@ -792,86 +792,86 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>600001</v>
+        <v>100001</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>VASO TALLADO BOSQUE</t>
+          <t>GIN BOSQUE NATIVO BOTELLA 500 ML</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CRISTALERIA</t>
+          <t>BEBIDAS</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>VIDRIO TALLADO</t>
+          <t>GIN</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3</v>
+        <v>760</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>7.6</v>
+        <v>2035.8</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>5</v>
+        <v>1276</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>12</v>
+        <v>3312</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>20</v>
+        <v>5347</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>12</v>
+        <v>2025</v>
       </c>
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>100001</v>
+        <v>600001</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>GIN BOSQUE NATIVO BOTELLA 500 ML</t>
+          <t>VASO TALLADO BOSQUE</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>BEBIDAS</t>
+          <t>CRISTALERIA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>GIN</t>
+          <t>VIDRIO TALLADO</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>980</v>
+        <v>3</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1978.5</v>
+        <v>7.6</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>998</v>
+        <v>5</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>2977</v>
+        <v>12</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4956</v>
+        <v>20</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>2025</v>
+        <v>12</v>
       </c>
       <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
@@ -896,22 +896,22 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>678</v>
+        <v>660</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>788.8</v>
+        <v>788.4</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>900</v>
+        <v>917</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1688</v>
+        <v>1705</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>46</v>
@@ -942,7 +942,7 @@
         <v>36</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>36.1</v>
+        <v>35.5</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>1</v>
@@ -951,10 +951,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>7</v>
@@ -964,11 +964,11 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>110005</v>
+        <v>100002</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA TEMPLE BLACK SOUL STOUT 473 ML</t>
+          <t>GIN BOSQUE ALTA MONTAÑA BOTELLA 500 ML</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -978,40 +978,38 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>CERVEZAS</t>
+          <t>GIN</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>6</v>
+        <v>538</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>4.9</v>
+        <v>424.2</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>4</v>
+        <v>310</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>18</v>
-      </c>
+        <v>735</v>
+      </c>
+      <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>100002</v>
+        <v>110005</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>GIN BOSQUE ALTA MONTAÑA BOTELLA 500 ML</t>
+          <t>CERVEZA TEMPLE BLACK SOUL STOUT 473 ML</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1021,28 +1019,30 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>GIN</t>
+          <t>CERVEZAS</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>554</v>
+        <v>6</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>424.2</v>
+        <v>4.4</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>294</v>
+        <v>3</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>719</v>
-      </c>
-      <c r="K13" s="2" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
     </row>
@@ -1066,22 +1066,22 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>2026</v>
+        <v>2002</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1036.1</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>2</v>
+        <v>1033.5</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>1.9</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>591</v>
@@ -1112,7 +1112,7 @@
         <v>19</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>9.6</v>
+        <v>9.4</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>2</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>10</v>
@@ -1155,10 +1155,10 @@
         <v>715</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>348.2</v>
+        <v>346.6</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
@@ -1196,7 +1196,7 @@
         <v>212</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>75</v>
+        <v>74.8</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>2.8</v>
@@ -1208,52 +1208,11 @@
         <v>0</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>500019</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>GIFT PACK NATIVO</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>COMBO</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>GIFT PACK</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>